<commit_message>
chore: checkpoint pending workspace changes
</commit_message>
<xml_diff>
--- a/sources/automations/中证红利信号/中证红利每日信号.xlsx
+++ b/sources/automations/中证红利信号/中证红利每日信号.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证红利每日信号" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中证红利每日信号'!$A$1:$P$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中证红利每日信号'!$A$1:$P$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2598,7 +2598,7 @@
       <c r="C37" s="4" t="n">
         <v>4.57</v>
       </c>
-      <c r="D37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="n"/>
       <c r="E37" s="3" t="inlineStr">
         <is>
           <t>2026-07-16</t>
@@ -2656,8 +2656,80 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>1.7404</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>2.859599999999999</v>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>未进入加大买入区间</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>4.38</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>12.26</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>6.12</t>
+        </is>
+      </c>
+      <c r="P38" s="7" t="inlineStr">
+        <is>
+          <t>理杏仁公开页面</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P37"/>
+  <autoFilter ref="A1:P38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: sync latest wiki and market tools
</commit_message>
<xml_diff>
--- a/sources/automations/中证红利信号/中证红利每日信号.xlsx
+++ b/sources/automations/中证红利信号/中证红利每日信号.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证红利每日信号" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中证红利每日信号'!$A$1:$P$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'中证红利每日信号'!$A$1:$P$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -3486,7 +3486,7 @@
       <c r="C51" s="4" t="n">
         <v>4.19</v>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="n"/>
       <c r="E51" s="3" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -3514,18 +3514,194 @@
           <t>历史分位点待验证，暂不判定加大买入区间</t>
         </is>
       </c>
-      <c r="L51" s="3" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr"/>
+      <c r="L51" s="3" t="n"/>
+      <c r="M51" s="4" t="n"/>
+      <c r="N51" s="4" t="n"/>
+      <c r="O51" s="4" t="n"/>
       <c r="P51" s="7" t="inlineStr">
         <is>
           <t>理杏仁待验证</t>
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D52" s="4" t="n"/>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>1.7114</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>2.4886</v>
+      </c>
+      <c r="H52" s="6" t="inlineStr"/>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>历史分位点待验证，暂不判定加大买入区间</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="n"/>
+      <c r="M52" s="4" t="n"/>
+      <c r="N52" s="4" t="n"/>
+      <c r="O52" s="4" t="n"/>
+      <c r="P52" s="7" t="inlineStr">
+        <is>
+          <t>理杏仁待验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>1.7074</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>2.4526</v>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr">
+        <is>
+          <t>历史分位点待验证，暂不判定加大买入区间</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="n"/>
+      <c r="M53" s="4" t="n"/>
+      <c r="N53" s="4" t="n"/>
+      <c r="O53" s="4" t="n"/>
+      <c r="P53" s="7" t="inlineStr">
+        <is>
+          <t>理杏仁待验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>4.18</v>
+      </c>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>1.7161</v>
+      </c>
+      <c r="G54" s="5" t="n">
+        <v>2.4639</v>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>未进入加大买入区间</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>4.26</t>
+        </is>
+      </c>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>7.04</t>
+        </is>
+      </c>
+      <c r="O54" s="4" t="inlineStr">
+        <is>
+          <t>6.11</t>
+        </is>
+      </c>
+      <c r="P54" s="7" t="inlineStr">
+        <is>
+          <t>理杏仁公开页面</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P51"/>
+  <autoFilter ref="A1:P54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>